<commit_message>
Stage 8 review fixes: D-011
</commit_message>
<xml_diff>
--- a/output/archive/QuenverellData/data/vp-b/rnaseq/processed/vp-b-covariate-model-interim-v2.xlsx
+++ b/output/archive/QuenverellData/data/vp-b/rnaseq/processed/vp-b-covariate-model-interim-v2.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sample QC" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data acceptance" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Covariate model" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model review" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
@@ -150,7 +150,7 @@
   <commentList>
     <comment ref="C4" authorId="0" shapeId="0">
       <text>
-        <t>Do not fit the covariate terms until the batch column is matched to the run log</t>
+        <t>Record outstanding metadata clarifications before releasing adjusted contrasts.</t>
       </text>
     </comment>
   </commentList>
@@ -163,9 +163,9 @@
     <author>Nadia Rahmani</author>
   </authors>
   <commentList>
-    <comment ref="D3" authorId="0" shapeId="0">
+    <comment ref="D2" authorId="0" shapeId="0">
       <text>
-        <t>Keep the sex term in until the metadata review; the decision on removing it has not been made</t>
+        <t>Confirm model specification against revised metadata before completing review.</t>
       </text>
     </comment>
   </commentList>
@@ -175,18 +175,12 @@
 <file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>Nadia Rahmani</author>
     <author>Dr E. Ostlund</author>
   </authors>
   <commentList>
-    <comment ref="F2" authorId="0" shapeId="0">
+    <comment ref="F3" authorId="0" shapeId="0">
       <text>
-        <t>Mark provisional where the batch column is not matched</t>
-      </text>
-    </comment>
-    <comment ref="A3" authorId="1" shapeId="0">
-      <text>
-        <t>Rows left blank until the model is refitted on the revised metadata</t>
+        <t>Leave final results blank until metadata reconciliation and model review are complete.</t>
       </text>
     </comment>
   </commentList>
@@ -606,7 +600,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Interim. Partial results only; final conclusions pending revised sample metadata from the client.</t>
+          <t>Interim. Count matrix accepted; covariate modelling and review remain open pending reconciliation of revised sample metadata.</t>
         </is>
       </c>
     </row>
@@ -664,31 +658,31 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Accepted for downstream use on 23/09/2026</t>
+          <t>Accepted for downstream analysis</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Library size</t>
+          <t>Revised sample metadata</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Accepted</t>
+          <t>Received</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>All libraries within the acceptance band in the analysis plan</t>
+          <t>Covariate modelling continuing; reconciliation remains open</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Sample sheet</t>
+          <t>Metadata reconciliation</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -698,33 +692,21 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Clinical fields incomplete for part of the cohort; revised sheet requested from the client</t>
+          <t>Outstanding clarifications to be recorded in the engagement metadata log</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Batch column</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Batch labels not yet matched to the sequencing run log</t>
-        </is>
-      </c>
+          <t>Model input review</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Donor pairing</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr"/>
       <c r="B6" s="2" t="inlineStr"/>
       <c r="C6" s="2" t="inlineStr"/>
     </row>
@@ -758,146 +740,102 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Term</t>
+          <t>Model component</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Condition</t>
+          <t>Clinical covariate specification</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Primary contrast</t>
+          <t>Engagement analysis plan</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Fitted</t>
+          <t>Under review</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Provisional until sample metadata is revised</t>
+          <t>Reconcile against revised sample metadata</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>Provisional contrasts</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Covariate</t>
+          <t>Interim analysis records</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Fitted</t>
+          <t>Provisional</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Provisional</t>
+          <t>Not released for final interpretation</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Age band</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Covariate</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Fitted</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Band boundaries as in the study plan</t>
-        </is>
-      </c>
+          <t>Final model terms</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Clinical response group</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Covariate</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Provisional</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Depends on revised sample sheet</t>
-        </is>
-      </c>
+          <t>Adjustment and diagnostics</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Collection batch</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Covariate</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Not fitted</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for batch labels</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Donor</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Random term</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Not fitted</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for donor pairing</t>
-        </is>
-      </c>
+      <c r="A7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -956,69 +894,45 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Condition, primary</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Dr A. Briand</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>23/09/2026</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Provisional</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Provisional</t>
-        </is>
-      </c>
+          <t>Provisional clinical covariate contrasts</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Interim only</t>
+          <t>See interim analysis records; review open</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Condition, adjusted for sex and age</t>
+          <t>Final adjusted contrasts</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr"/>
       <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Pending metadata reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Clinical response group</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr"/>
       <c r="B4" s="2" t="inlineStr"/>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Blocked on revised sample sheet</t>
-        </is>
-      </c>
+      <c r="F4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Condition, batch-adjusted</t>
-        </is>
-      </c>
+      <c r="A5" s="2" t="inlineStr"/>
       <c r="B5" s="2" t="inlineStr"/>
       <c r="C5" s="2" t="inlineStr"/>
       <c r="D5" s="2" t="inlineStr"/>

</xml_diff>